<commit_message>
Update service image styles and push latest services spreadsheet
</commit_message>
<xml_diff>
--- a/public/services.xlsx
+++ b/public/services.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\khano\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\For Other\fehed\Tech\TechInnoSphere-Single\TechInnoSphere\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{102186CA-0FE6-4357-9B07-1BC71079C1CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{815F4279-9215-41CA-A724-56C7A83625CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -340,46 +340,46 @@
     <t>Assess Security</t>
   </si>
   <si>
-    <t>https://drive.google.com/file/d/18dJ_SOXO7QU-iKWORelboom02c6YkUAa/view?usp=drive_link</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1p7lrs6YvMamsppBj59z7VUWU-NwQaoNs/view?usp=drive_link</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1sA74qDS2DrdhnP2qXaU2KX5z_bKA4gVm/view?usp=drive_link</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/16f4Ay7uwGobEoM1LKwjb72z8LXexAdGh/view?usp=drive_link</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/10rq0qgW0RkfnBpRXe4XjPKqO5WZix0FN/view?usp=drive_link</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1F-M-kwRRLIpFB15eXWRR6-EYj4VBw3Ps/view?usp=sharing</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1YNuBVtKDxXOnha7BYRrYrjSh16uWLxpy/view?usp=sharing</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1Y7UFHgwETXnz8yO4aWpCi8uyFbBWvND-/view?usp=sharing</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1Qcn_XcoL84SxbrxfFg3JyILiavrQVAdd/view?usp=sharing</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1qePk37XFzO7Gp-P3snk-J04aiFficu7x/view?usp=sharing</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1EFMradLdMOm8Y5JeL1e7dR66ebWxbKGX/view?usp=sharing</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1K2LpwT7_S0onrpRevvym3-yIUFWaXrI7/view?usp=sharing</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1q78XjlD3jZ22Y8b4XHfeVo7wmTmIQ57Z/view?usp=sharing</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1H5icgTFTA0SmP-75TcAOkd-p1xcB-WW7/view?usp=sharing</t>
+    <t>https://drive.google.com/uc?export=view&amp;id=18dJ_SOXO7QU-iKWORelboom02c6YkUAa</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/uc?export=view&amp;id=1p7lrs6YvMamsppBj59z7VUWU-NwQaoNs</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/uc?export=view&amp;id=1sA74qDS2DrdhnP2qXaU2KX5z_bKA4gVm</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/uc?export=view&amp;id=16f4Ay7uwGobEoM1LKwjb72z8LXexAdGh</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/uc?export=view&amp;id=10rq0qgW0RkfnBpRXe4XjPKqO5WZix0FN</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/uc?export=view&amp;id=1F-M-kwRRLIpFB15eXWRR6-EYj4VBw3Ps</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/uc?export=view&amp;id=1YNuBVtKDxXOnha7BYRrYrjSh16uWLxpy</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/uc?export=view&amp;id=1Y7UFHgwETXnz8yO4aWpCi8uyFbBWvND-</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/uc?export=view&amp;id=1Qcn_XcoL84SxbrxfFg3JyILiavrQVAdd</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/uc?export=view&amp;id=1qePk37XFzO7Gp-P3snk-J04aiFficu7x</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/uc?export=view&amp;id=1EFMradLdMOm8Y5JeL1e7dR66ebWxbKGX</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/uc?export=view&amp;id=1K2LpwT7_S0onrpRevvym3-yIUFWaXrI7</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/uc?export=view&amp;id=1q78XjlD3jZ22Y8b4XHfeVo7wmTmIQ57Z</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/uc?export=view&amp;id=1H5icgTFTA0SmP-75TcAOkd-p1xcB-WW7</t>
   </si>
 </sst>
 </file>
@@ -768,13 +768,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35.09765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.8984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="142.796875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="81.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -806,7 +808,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -838,7 +840,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -870,7 +872,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -902,7 +904,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>33</v>
       </c>
@@ -934,7 +936,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>40</v>
       </c>
@@ -966,7 +968,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>47</v>
       </c>
@@ -998,7 +1000,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>54</v>
       </c>
@@ -1030,7 +1032,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>61</v>
       </c>
@@ -1062,7 +1064,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>67</v>
       </c>
@@ -1094,7 +1096,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>74</v>
       </c>
@@ -1126,7 +1128,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>80</v>
       </c>
@@ -1158,7 +1160,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>87</v>
       </c>
@@ -1190,7 +1192,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>93</v>
       </c>
@@ -1222,7 +1224,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>100</v>
       </c>
@@ -1255,14 +1257,6 @@
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" xr:uid="{8517208E-4677-4571-BFB8-EA5F7B311D83}"/>
-    <hyperlink ref="D3" r:id="rId2" xr:uid="{002842D8-991B-4D7B-906F-C1971B9065A6}"/>
-    <hyperlink ref="D4" r:id="rId3" xr:uid="{AE0C29E5-838D-4C1D-A7C4-AA8EBFE123A0}"/>
-    <hyperlink ref="D5" r:id="rId4" xr:uid="{464D632C-2781-4AAB-AFC7-359528CE089C}"/>
-    <hyperlink ref="D6" r:id="rId5" xr:uid="{68914291-5F2F-4DCD-9434-F921D1ACBEF4}"/>
-    <hyperlink ref="D7" r:id="rId6" xr:uid="{D92ABB58-541B-4DEF-A3F2-423E91471449}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError sqref="A1:J1 A15:C15 A2:C2 E2:J2 A3:C3 E3:J3 A4:C4 E4:J4 A5:C5 E5:J5 A6:C6 E6:J6 A7:C7 E7:J7 A8:C8 E8:J8 A9:C9 E9:J9 A10:C10 E10:J10 A11:C11 E11:J11 A12:C12 E12:J12 A13:C13 E13:J13 A14:C14 E14:J14 E15:J15" numberStoredAsText="1"/>

</xml_diff>